<commit_message>
chore: actualizar calendario — eliminar revisión técnica, agregar artículo simulación ejecutiva, columna validación agente
</commit_message>
<xml_diff>
--- a/calendario-editorial-jun-jul-2026.xlsx
+++ b/calendario-editorial-jun-jul-2026.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="28">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -186,8 +186,22 @@
       <color rgb="00555555"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001E6B1E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E6B1E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -257,6 +271,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCEBEB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -330,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -493,6 +512,16 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -858,7 +887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -872,6 +901,7 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -889,12 +919,13 @@
       <c r="H1" s="46" t="n"/>
       <c r="I1" s="46" t="n"/>
       <c r="J1" s="46" t="n"/>
-      <c r="K1" s="47" t="n"/>
+      <c r="K1" s="46" t="n"/>
+      <c r="L1" s="47" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 2026-06-12  |  Anti-canibalización: verificado contra blog  |  Reglas de negocio: aplicadas  |  3 publicados · 17 listos · 2 descartados</t>
+          <t>Generado: 2026-06-12 | Actualizado: 2026-06-15 — revisión técnica agente aplicada | 3 publicados · 17 listos · 2 descartados</t>
         </is>
       </c>
       <c r="B2" s="46" t="n"/>
@@ -906,7 +937,8 @@
       <c r="H2" s="46" t="n"/>
       <c r="I2" s="46" t="n"/>
       <c r="J2" s="46" t="n"/>
-      <c r="K2" s="47" t="n"/>
+      <c r="K2" s="46" t="n"/>
+      <c r="L2" s="47" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -962,6 +994,11 @@
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Estado</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Validación Agente</t>
         </is>
       </c>
     </row>
@@ -980,7 +1017,8 @@
       <c r="H4" s="46" t="n"/>
       <c r="I4" s="46" t="n"/>
       <c r="J4" s="46" t="n"/>
-      <c r="K4" s="47" t="n"/>
+      <c r="K4" s="46" t="n"/>
+      <c r="L4" s="47" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="n">
@@ -1036,6 +1074,11 @@
           <t>♻ Reemplaza post sep-2025</t>
         </is>
       </c>
+      <c r="L5" s="56" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="12" t="n">
@@ -1091,9 +1134,14 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L6" s="56" t="inlineStr">
+        <is>
+          <t>✅ Verificado — eliminado "app-drivers" como perfil; meta y CTAs corregidos</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="12" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1101,49 +1149,54 @@
           <t>Jun S2</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Revisión técnica Chile 2026: dónde, costos y qué revisan</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>revisión técnica Chile 2026</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>~900</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Cómo simular un crédito automotriz con una ejecutiva real</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>cómo simular crédito automotriz</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>~250</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>~18</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>Conducción</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>C5</t>
-        </is>
-      </c>
-      <c r="I7" s="9" t="inlineStr">
-        <is>
-          <t>Normativa/evergreen</t>
-        </is>
-      </c>
-      <c r="J7" s="17" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Crédito Automotriz</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>Satélite educativo</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K7" s="16" t="inlineStr">
         <is>
           <t>📝 Listo</t>
+        </is>
+      </c>
+      <c r="L7" s="57" t="inlineStr">
+        <is>
+          <t>✅ Nuevo jun-2026 — ejecutiva real por WhatsApp; sin simulador automático; 0 errores de regla</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1215,8 @@
       <c r="H8" s="46" t="n"/>
       <c r="I8" s="46" t="n"/>
       <c r="J8" s="46" t="n"/>
-      <c r="K8" s="47" t="n"/>
+      <c r="K8" s="46" t="n"/>
+      <c r="L8" s="47" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="n">
@@ -1218,6 +1272,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L9" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="12" t="n">
@@ -1273,6 +1332,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L10" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -1326,6 +1390,11 @@
       <c r="K11" s="16" t="inlineStr">
         <is>
           <t>📝 Listo</t>
+        </is>
+      </c>
+      <c r="L11" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1413,8 @@
       <c r="H12" s="46" t="n"/>
       <c r="I12" s="46" t="n"/>
       <c r="J12" s="46" t="n"/>
-      <c r="K12" s="47" t="n"/>
+      <c r="K12" s="46" t="n"/>
+      <c r="L12" s="47" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="n">
@@ -1400,6 +1470,11 @@
           <t>🔧 Update Webflow</t>
         </is>
       </c>
+      <c r="L13" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="12" t="n">
@@ -1453,6 +1528,11 @@
       <c r="K14" s="16" t="inlineStr">
         <is>
           <t>📝 Listo</t>
+        </is>
+      </c>
+      <c r="L14" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1551,8 @@
       <c r="H15" s="46" t="n"/>
       <c r="I15" s="46" t="n"/>
       <c r="J15" s="46" t="n"/>
-      <c r="K15" s="47" t="n"/>
+      <c r="K15" s="46" t="n"/>
+      <c r="L15" s="47" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="n">
@@ -1527,6 +1608,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L16" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="12" t="n">
@@ -1582,6 +1668,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L17" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="n">
@@ -1637,6 +1728,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L18" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="12" t="n">
@@ -1690,6 +1786,11 @@
       <c r="K19" s="16" t="inlineStr">
         <is>
           <t>📝 Listo</t>
+        </is>
+      </c>
+      <c r="L19" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1809,8 @@
       <c r="H20" s="46" t="n"/>
       <c r="I20" s="46" t="n"/>
       <c r="J20" s="46" t="n"/>
-      <c r="K20" s="47" t="n"/>
+      <c r="K20" s="46" t="n"/>
+      <c r="L20" s="47" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -1764,6 +1866,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L21" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="12" t="n">
@@ -1819,6 +1926,11 @@
           <t>✅ Publicado 11-jun</t>
         </is>
       </c>
+      <c r="L22" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="5" t="n">
@@ -1872,6 +1984,11 @@
       <c r="K23" s="10" t="inlineStr">
         <is>
           <t>✅ Publicado jun-2026</t>
+        </is>
+      </c>
+      <c r="L23" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1921,6 +2038,11 @@
       <c r="K24" s="22" t="inlineStr">
         <is>
           <t>⚠ DESCARTADO — viola regla negocio</t>
+        </is>
+      </c>
+      <c r="L24" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1939,7 +2061,8 @@
       <c r="H25" s="46" t="n"/>
       <c r="I25" s="46" t="n"/>
       <c r="J25" s="46" t="n"/>
-      <c r="K25" s="47" t="n"/>
+      <c r="K25" s="46" t="n"/>
+      <c r="L25" s="47" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="5" t="n">
@@ -1995,6 +2118,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L26" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="12" t="n">
@@ -2050,6 +2178,11 @@
           <t>🔧 Esperar datos ANAC (3–10 jul)</t>
         </is>
       </c>
+      <c r="L27" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="5" t="n">
@@ -2105,6 +2238,11 @@
           <t>✅ Publicado jun-2026</t>
         </is>
       </c>
+      <c r="L28" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="12" t="n">
@@ -2158,6 +2296,11 @@
       <c r="K29" s="16" t="inlineStr">
         <is>
           <t>📝 Listo</t>
+        </is>
+      </c>
+      <c r="L29" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2319,8 @@
       <c r="H30" s="46" t="n"/>
       <c r="I30" s="46" t="n"/>
       <c r="J30" s="46" t="n"/>
-      <c r="K30" s="47" t="n"/>
+      <c r="K30" s="46" t="n"/>
+      <c r="L30" s="47" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="5" t="n">
@@ -2232,6 +2376,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L31" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="12" t="n">
@@ -2287,6 +2436,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L32" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="5" t="n">
@@ -2342,6 +2496,11 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L33" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="12" t="n">
@@ -2397,19 +2556,24 @@
           <t>📝 Listo</t>
         </is>
       </c>
+      <c r="L34" s="58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:K3"/>
   <mergeCells count="9">
-    <mergeCell ref="A12:K12"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A30:K30"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="A30:L30"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A12:L12"/>
+    <mergeCell ref="A4:L4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3457,7 +3621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3809,6 +3973,81 @@
       <c r="C27" s="31" t="inlineStr">
         <is>
           <t>BYD Dolphin publicado + pilar eléctricos Jul S4</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="59" t="inlineStr">
+        <is>
+          <t>Validación de borradores — jun 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Artículo Chevrolet Sail (C4)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>✅ Verificado</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Consumo en ciudad corregido (era valor mixto); 0 errores críticos; pendiente verificar LTZ 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Artículo Crédito Entre Particulares (C9/C1)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>✅ Verificado</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Género "ejecutiva" corregido (1 instancia); CTA corregido</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Artículo Crédito Sin Acreditar Ingresos (C2)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>✅ Verificado</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Eliminados "app-drivers" del perfil objetivo (regla crítica); meta y CTAs corregidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Artículo Simulador / Cómo simular (C2) — NUEVO</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>✅ Verificado</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Nuevo artículo reemplaza premisa de simulador automático; ejecutiva real por WhatsApp</t>
         </is>
       </c>
     </row>
@@ -6311,6 +6550,11 @@
           <t>SEMRUSH STATS — unidadcreditos.cl (CL) | Actualizado jun-2026</t>
         </is>
       </c>
+      <c r="B1" s="46" t="n"/>
+      <c r="C1" s="46" t="n"/>
+      <c r="D1" s="46" t="n"/>
+      <c r="E1" s="46" t="n"/>
+      <c r="F1" s="47" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -6318,6 +6562,11 @@
           <t>Fuente: Semrush · Base de datos Chile · Ordenado por tráfico estimado mensual</t>
         </is>
       </c>
+      <c r="B2" s="46" t="n"/>
+      <c r="C2" s="46" t="n"/>
+      <c r="D2" s="46" t="n"/>
+      <c r="E2" s="46" t="n"/>
+      <c r="F2" s="47" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -6325,6 +6574,11 @@
           <t>📊 RESUMEN DOMINIO: Rank Chile #2.269 | Organic Keywords: 6.188 | Tráfico orgánico estimado: 42.658 visitas/mes</t>
         </is>
       </c>
+      <c r="B3" s="46" t="n"/>
+      <c r="C3" s="46" t="n"/>
+      <c r="D3" s="46" t="n"/>
+      <c r="E3" s="46" t="n"/>
+      <c r="F3" s="47" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -7066,6 +7320,11 @@
           <t>INSIGHTS ESTRATÉGICOS — jun 2026</t>
         </is>
       </c>
+      <c r="B34" s="46" t="n"/>
+      <c r="C34" s="46" t="n"/>
+      <c r="D34" s="46" t="n"/>
+      <c r="E34" s="46" t="n"/>
+      <c r="F34" s="47" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="34" t="inlineStr">
@@ -7078,6 +7337,10 @@
           <t>Gasolineras + UTM = 80,8% del tráfico orgánico total. Ninguno de los dos convierte a crédito automotriz. El calendario jun-jul apunta a construir tráfico en clusters de conversión.</t>
         </is>
       </c>
+      <c r="C35" s="46" t="n"/>
+      <c r="D35" s="46" t="n"/>
+      <c r="E35" s="46" t="n"/>
+      <c r="F35" s="47" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="35" t="inlineStr">
@@ -7090,6 +7353,10 @@
           <t>Los artículos de jun-2026 (BYD Dolphin, Batería, Neblina) fueron publicados hace pocos días — Semrush demora 2–4 semanas en indexar posiciones nuevas. Verificar en la próxima revisión semanal.</t>
         </is>
       </c>
+      <c r="C36" s="46" t="n"/>
+      <c r="D36" s="46" t="n"/>
+      <c r="E36" s="46" t="n"/>
+      <c r="F36" s="47" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="34" t="inlineStr">
@@ -7102,6 +7369,10 @@
           <t>/post/que-es-un-credito-automotriz no aparece en el top 50 por tráfico. El brief actualizado debe reemplazar el post existente de sep-2025 para recuperar posiciones.</t>
         </is>
       </c>
+      <c r="C37" s="46" t="n"/>
+      <c r="D37" s="46" t="n"/>
+      <c r="E37" s="46" t="n"/>
+      <c r="F37" s="47" t="n"/>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="35" t="inlineStr">
@@ -7114,6 +7385,10 @@
           <t>3 artículos de Registro Civil/patentes en top 20 con alta cobertura (273–195 keywords) — cluster C9 bien posicionado. Los nuevos artículos de transferencia y prenda enlazarán a estos.</t>
         </is>
       </c>
+      <c r="C38" s="46" t="n"/>
+      <c r="D38" s="46" t="n"/>
+      <c r="E38" s="46" t="n"/>
+      <c r="F38" s="47" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="34" t="inlineStr">
@@ -7126,6 +7401,10 @@
           <t>Ningún artículo del top 50 presenta caída de posición verificada por ≥4 semanas. No reescribir. Monitorear en revisión semanal de los lunes.</t>
         </is>
       </c>
+      <c r="C39" s="46" t="n"/>
+      <c r="D39" s="46" t="n"/>
+      <c r="E39" s="46" t="n"/>
+      <c r="F39" s="47" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:F4"/>

</xml_diff>

<commit_message>
calendario: adelantar #24 alertas seguridad a Jul S1
- Artículo 'Cómo verificar si un auto tiene alertas de seguridad
  pendientes en Chile' movido de Jul S4 → Jul S1 (semana 7-13 jul)
- Trigger: alerta SERNAC Jeep Grand Cherokee (232 unidades,
  feb 2023–dic 2025, reposacabezas 2a fila)
- Agregar bloque de actualidad con link a sernac.cl al publicar
</commit_message>
<xml_diff>
--- a/calendario-editorial-jun-jul-2026.xlsx
+++ b/calendario-editorial-jun-jul-2026.xlsx
@@ -887,7 +887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2559,6 +2559,66 @@
       <c r="L34" s="58" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="B35" s="20" t="inlineStr">
+        <is>
+          <t>Jul S1</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Cómo verificar si un auto tiene alertas de seguridad pendientes en Chile</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>alerta de seguridad auto Chile</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>~20</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>~15</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>Comprar Auto</t>
+        </is>
+      </c>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="I35" s="15" t="inlineStr">
+        <is>
+          <t>Guía verificación</t>
+        </is>
+      </c>
+      <c r="J35" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K35" s="16" t="inlineStr">
+        <is>
+          <t>📝 Listo</t>
+        </is>
+      </c>
+      <c r="L35" s="58" t="inlineStr">
+        <is>
+          <t>✅ Nuevo jun-2026 — portal ANAC; 30+ marcas; gratuito para todos los dueños; 0 errores de regla | ⚡ Adelantado a Jul S1: alerta SERNAC Jeep Grand Cherokee (232–247 unidades, feb 2023–dic 2025) — agregar bloque de actualidad con link a sernac.cl</t>
         </is>
       </c>
     </row>

</xml_diff>